<commit_message>
Scrap quotidien automatique (2026-09-13)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1072</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1082</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1072"/>
+  <dimension ref="A1:K1082"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50859,8 +50859,478 @@
         <v>36893901</v>
       </c>
     </row>
+    <row r="1073">
+      <c r="A1073" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1073" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1073" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1073" t="inlineStr">
+        <is>
+          <t>2/36</t>
+        </is>
+      </c>
+      <c r="I1073" s="4" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="J1073" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1073" t="n">
+        <v>36323282</v>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>Guided Session (English version)</t>
+        </is>
+      </c>
+      <c r="E1074" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1074" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1074" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1074" t="inlineStr">
+        <is>
+          <t>13/18</t>
+        </is>
+      </c>
+      <c r="I1074" s="5" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="J1074" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1074" t="n">
+        <v>36323128</v>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1075" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1075" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1075" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1075" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1075" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1075" t="n">
+        <v>38771780</v>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1076" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1076" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1076" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I1076" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J1076" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1076" t="n">
+        <v>36329210</v>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1077" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1077" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1077" t="inlineStr">
+        <is>
+          <t>14/36</t>
+        </is>
+      </c>
+      <c r="I1077" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1077" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1077" t="n">
+        <v>38771880</v>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1078" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1078" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1078" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1078" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1078" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1078" t="n">
+        <v>36329975</v>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1079" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1079" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1079" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
+      <c r="I1079" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="J1079" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1079" t="n">
+        <v>42468534</v>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1080" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1080" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1080" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1080" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1080" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1080" t="n">
+        <v>42468535</v>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1081" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1081" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1081" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1081" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1081" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1081" t="n">
+        <v>36323867</v>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1082" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1082" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1082" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="I1082" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J1082" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1082" t="n">
+        <v>42468555</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1072"/>
+  <autoFilter ref="A1:K1082"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-14)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1082</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1090</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1082"/>
+  <dimension ref="A1:K1090"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50367,18 +50367,18 @@
         </is>
       </c>
       <c r="F1062" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G1062" t="n">
         <v>10</v>
       </c>
       <c r="H1062" t="inlineStr">
         <is>
-          <t>9/10</t>
-        </is>
-      </c>
-      <c r="I1062" s="3" t="n">
-        <v>90</v>
+          <t>7/10</t>
+        </is>
+      </c>
+      <c r="I1062" s="5" t="n">
+        <v>70</v>
       </c>
       <c r="J1062" t="inlineStr">
         <is>
@@ -51329,8 +51329,384 @@
         <v>42468555</v>
       </c>
     </row>
+    <row r="1083">
+      <c r="A1083" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1083" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1083" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1083" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1083" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1083" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1083" t="n">
+        <v>37240292</v>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1084" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1084" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1084" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1084" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1084" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1084" t="n">
+        <v>36336038</v>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1085" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1085" t="n">
+        <v>19</v>
+      </c>
+      <c r="G1085" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1085" t="inlineStr">
+        <is>
+          <t>19/36</t>
+        </is>
+      </c>
+      <c r="I1085" s="5" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="J1085" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1085" t="n">
+        <v>37240435</v>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1086" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1086" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1086" t="inlineStr">
+        <is>
+          <t>21/36</t>
+        </is>
+      </c>
+      <c r="I1086" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J1086" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1086" t="n">
+        <v>36892152</v>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1087" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1087" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1087" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I1087" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J1087" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1087" t="n">
+        <v>36336253</v>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1088" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1088" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1088" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1088" t="inlineStr">
+        <is>
+          <t>26/28</t>
+        </is>
+      </c>
+      <c r="I1088" s="3" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="J1088" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1088" t="n">
+        <v>36692765</v>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1089" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1089" t="n">
+        <v>35</v>
+      </c>
+      <c r="G1089" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1089" t="inlineStr">
+        <is>
+          <t>35/34</t>
+        </is>
+      </c>
+      <c r="I1089" s="3" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="J1089" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1089" t="n">
+        <v>42480968</v>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1090" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1090" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1090" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1090" t="inlineStr">
+        <is>
+          <t>10/36</t>
+        </is>
+      </c>
+      <c r="I1090" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1090" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1090" t="n">
+        <v>36892107</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1082"/>
+  <autoFilter ref="A1:K1090"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-15)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1090</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1097</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1090"/>
+  <dimension ref="A1:K1097"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51705,8 +51705,337 @@
         <v>36892107</v>
       </c>
     </row>
+    <row r="1091">
+      <c r="A1091" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1091" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1091" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1091" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1091" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I1091" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J1091" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1091" t="n">
+        <v>36390339</v>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1092" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1092" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1092" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I1092" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J1092" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1092" t="n">
+        <v>36281142</v>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1093" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1093" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1093" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="I1093" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J1093" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1093" t="n">
+        <v>38531918</v>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1094" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1094" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1094" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I1094" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1094" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1094" t="n">
+        <v>36928737</v>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1095" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1095" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1095" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I1095" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J1095" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1095" t="n">
+        <v>36281006</v>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1096" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1096" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1096" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1096" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1096" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1096" t="n">
+        <v>37873148</v>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1097" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1097" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1097" t="inlineStr">
+        <is>
+          <t>15/36</t>
+        </is>
+      </c>
+      <c r="I1097" s="4" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="J1097" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1097" t="n">
+        <v>36929043</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1090"/>
+  <autoFilter ref="A1:K1097"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-16)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1097</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1097"/>
+  <dimension ref="A1:K1104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52034,8 +52034,337 @@
         <v>36929043</v>
       </c>
     </row>
+    <row r="1098">
+      <c r="A1098" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F1098" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1098" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1098" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1098" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1098" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1098" t="n">
+        <v>36321370</v>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1099" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1099" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1099" t="inlineStr">
+        <is>
+          <t>4/28</t>
+        </is>
+      </c>
+      <c r="I1099" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1099" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1099" t="n">
+        <v>40188421</v>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1100" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1100" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1100" t="inlineStr">
+        <is>
+          <t>3/18</t>
+        </is>
+      </c>
+      <c r="I1100" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1100" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1100" t="n">
+        <v>36929169</v>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1101" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1101" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1101" t="inlineStr">
+        <is>
+          <t>3/18</t>
+        </is>
+      </c>
+      <c r="I1101" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1101" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1101" t="n">
+        <v>36298249</v>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1102" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1102" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1102" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1102" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I1102" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J1102" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1102" t="n">
+        <v>36297694</v>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1103" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1103" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1103" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1103" t="inlineStr">
+        <is>
+          <t>14/28</t>
+        </is>
+      </c>
+      <c r="I1103" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1103" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1103" t="n">
+        <v>36298056</v>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1104" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1104" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1104" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1104" t="inlineStr">
+        <is>
+          <t>11/36</t>
+        </is>
+      </c>
+      <c r="I1104" s="4" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="J1104" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1104" t="n">
+        <v>40188452</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1097"/>
+  <autoFilter ref="A1:K1104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-18)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1124</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1104"/>
+  <dimension ref="A1:K1124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52363,8 +52363,948 @@
         <v>40188452</v>
       </c>
     </row>
+    <row r="1105">
+      <c r="A1105" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1105" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1105" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1105" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1105" t="inlineStr">
+        <is>
+          <t>4/28</t>
+        </is>
+      </c>
+      <c r="I1105" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1105" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1105" t="n">
+        <v>36321419</v>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1106" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1106" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1106" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1106" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I1106" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J1106" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1106" t="n">
+        <v>36929301</v>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1107" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1107" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1107" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I1107" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1107" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1107" t="n">
+        <v>36298350</v>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F1108" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1108" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1108" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1108" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1108" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1108" t="n">
+        <v>36298391</v>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1109" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1109" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1109" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I1109" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J1109" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1109" t="n">
+        <v>36298588</v>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1110" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1110" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1110" t="inlineStr">
+        <is>
+          <t>22/36</t>
+        </is>
+      </c>
+      <c r="I1110" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J1110" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1110" t="n">
+        <v>40189910</v>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F1111" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1111" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1111" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1111" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1111" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1111" t="n">
+        <v>37090015</v>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1112" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1112" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1112" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1112" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1112" t="n">
+        <v>42435195</v>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1113" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1113" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1113" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1113" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1113" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1113" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1113" t="n">
+        <v>42435130</v>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1114" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1114" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1114" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1114" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1114" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1114" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1114" t="n">
+        <v>37230123</v>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1115" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1115" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1115" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1115" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1115" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1115" t="n">
+        <v>37230159</v>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1116" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1116" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1116" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1116" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1116" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1116" t="n">
+        <v>37090973</v>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1117" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1117" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1117" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1117" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1117" t="n">
+        <v>42430590</v>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1118" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1118" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1118" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1118" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1118" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1118" t="n">
+        <v>42431393</v>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1119" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1119" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1119" t="inlineStr">
+        <is>
+          <t>14/28</t>
+        </is>
+      </c>
+      <c r="I1119" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1119" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1119" t="n">
+        <v>36321570</v>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1120" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1120" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1120" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I1120" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1120" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1120" t="n">
+        <v>36929392</v>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1121" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1121" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1121" t="inlineStr">
+        <is>
+          <t>2/18</t>
+        </is>
+      </c>
+      <c r="I1121" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J1121" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1121" t="n">
+        <v>36298765</v>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1122" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1122" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1122" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1122" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1122" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1122" t="n">
+        <v>36298819</v>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1123" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1123" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1123" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1123" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1123" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1123" t="n">
+        <v>36298872</v>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1124" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1124" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1124" t="inlineStr">
+        <is>
+          <t>13/34</t>
+        </is>
+      </c>
+      <c r="I1124" s="4" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="J1124" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1124" t="n">
+        <v>40190139</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1104"/>
+  <autoFilter ref="A1:K1124"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-19)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1132</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1124"/>
+  <dimension ref="A1:K1132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -53303,8 +53303,384 @@
         <v>40190139</v>
       </c>
     </row>
+    <row r="1125">
+      <c r="A1125" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1125" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1125" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1125" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="I1125" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1125" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1125" t="n">
+        <v>36319508</v>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1126" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1126" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1126" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1126" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1126" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1126" t="n">
+        <v>42666072</v>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1127" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1127" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1127" t="inlineStr">
+        <is>
+          <t>2/18</t>
+        </is>
+      </c>
+      <c r="I1127" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J1127" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1127" t="n">
+        <v>36320065</v>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1128" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1128" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I1128" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1128" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1128" t="n">
+        <v>36320666</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F1129" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1129" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1129" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I1129" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1129" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1129" t="n">
+        <v>36320789</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1130" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1130" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1130" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I1130" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J1130" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1130" t="n">
+        <v>36320899</v>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1131" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1131" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1131" t="inlineStr">
+        <is>
+          <t>29/36</t>
+        </is>
+      </c>
+      <c r="I1131" s="5" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="J1131" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1131" t="n">
+        <v>36893836</v>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1132" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1132" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1132" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1132" t="inlineStr">
+        <is>
+          <t>9/36</t>
+        </is>
+      </c>
+      <c r="I1132" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1132" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1132" t="n">
+        <v>36893903</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1124"/>
+  <autoFilter ref="A1:K1132"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-20)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1140</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1132"/>
+  <dimension ref="A1:K1140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -53679,8 +53679,384 @@
         <v>36893903</v>
       </c>
     </row>
+    <row r="1133">
+      <c r="A1133" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1133" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1133" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1133" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1133" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1133" t="n">
+        <v>36323283</v>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>Guided Session (English version)</t>
+        </is>
+      </c>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1134" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1134" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1134" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I1134" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J1134" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1134" t="n">
+        <v>36323129</v>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1135" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1135" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1135" t="inlineStr">
+        <is>
+          <t>7/36</t>
+        </is>
+      </c>
+      <c r="I1135" s="4" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="J1135" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1135" t="n">
+        <v>38771781</v>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1136" t="n">
+        <v>19</v>
+      </c>
+      <c r="G1136" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1136" t="inlineStr">
+        <is>
+          <t>19/28</t>
+        </is>
+      </c>
+      <c r="I1136" s="5" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="J1136" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1136" t="n">
+        <v>36329211</v>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1137" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1137" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1137" t="inlineStr">
+        <is>
+          <t>26/36</t>
+        </is>
+      </c>
+      <c r="I1137" s="5" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="J1137" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1137" t="n">
+        <v>38771881</v>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1138" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1138" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1138" t="inlineStr">
+        <is>
+          <t>17/28</t>
+        </is>
+      </c>
+      <c r="I1138" s="5" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="J1138" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1138" t="n">
+        <v>36329976</v>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1139" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1139" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1139" t="inlineStr">
+        <is>
+          <t>27/36</t>
+        </is>
+      </c>
+      <c r="I1139" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1139" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1139" t="n">
+        <v>36323868</v>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1140" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1140" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1140" t="inlineStr">
+        <is>
+          <t>14/36</t>
+        </is>
+      </c>
+      <c r="I1140" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1140" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1140" t="n">
+        <v>36935883</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1132"/>
+  <autoFilter ref="A1:K1140"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-21)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1148</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1140"/>
+  <dimension ref="A1:K1148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54055,8 +54055,384 @@
         <v>36935883</v>
       </c>
     </row>
+    <row r="1141">
+      <c r="A1141" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1141" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1141" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>11/36</t>
+        </is>
+      </c>
+      <c r="I1141" s="4" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="J1141" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1141" t="n">
+        <v>37240293</v>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1142" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1142" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1142" t="inlineStr">
+        <is>
+          <t>22/28</t>
+        </is>
+      </c>
+      <c r="I1142" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J1142" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1142" t="n">
+        <v>36336039</v>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1143" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1143" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>9/36</t>
+        </is>
+      </c>
+      <c r="I1143" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1143" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1143" t="n">
+        <v>37240436</v>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1144" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1144" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>12/36</t>
+        </is>
+      </c>
+      <c r="I1144" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1144" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1144" t="n">
+        <v>36892153</v>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1145" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1145" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1145" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1145" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1145" t="n">
+        <v>36336254</v>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1146" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1146" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1146" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1146" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1146" t="n">
+        <v>36692766</v>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1147" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1147" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>38/36</t>
+        </is>
+      </c>
+      <c r="I1147" s="3" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="J1147" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1147" t="n">
+        <v>42481094</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1148" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1148" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>18/36</t>
+        </is>
+      </c>
+      <c r="I1148" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1148" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1148" t="n">
+        <v>36892108</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1140"/>
+  <autoFilter ref="A1:K1148"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-22)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1148"/>
+  <dimension ref="A1:K1156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54431,8 +54431,384 @@
         <v>36892108</v>
       </c>
     </row>
+    <row r="1149">
+      <c r="A1149" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1149" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1149" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1149" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1149" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1149" t="n">
+        <v>36390340</v>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1150" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1150" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1150" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1150" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1150" t="n">
+        <v>36281143</v>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1151" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1151" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>3/18</t>
+        </is>
+      </c>
+      <c r="I1151" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1151" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1151" t="n">
+        <v>38531919</v>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1152" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1152" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I1152" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1152" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1152" t="n">
+        <v>36928738</v>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1153" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1153" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>9/12</t>
+        </is>
+      </c>
+      <c r="I1153" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1153" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1153" t="n">
+        <v>43010262</v>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F1154" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1154" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1154" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1154" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1154" t="n">
+        <v>36281007</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F1155" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1155" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I1155" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J1155" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1155" t="n">
+        <v>37873149</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1156" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1156" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>17/36</t>
+        </is>
+      </c>
+      <c r="I1156" s="4" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="J1156" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1156" t="n">
+        <v>36929044</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1148"/>
+  <autoFilter ref="A1:K1156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-23)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1156"/>
+  <dimension ref="A1:K1164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54807,8 +54807,384 @@
         <v>36929044</v>
       </c>
     </row>
+    <row r="1157">
+      <c r="A1157" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1157" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1157" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1157" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1157" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1157" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1157" t="n">
+        <v>36321371</v>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1158" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1158" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1158" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1158" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1158" t="n">
+        <v>40188422</v>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1159" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1159" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I1159" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1159" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1159" t="n">
+        <v>36929170</v>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1160" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1160" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1160" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I1160" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1160" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1160" t="n">
+        <v>36298250</v>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1161" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1161" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1161" t="inlineStr">
+        <is>
+          <t>7/12</t>
+        </is>
+      </c>
+      <c r="I1161" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J1161" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1161" t="n">
+        <v>43010263</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F1162" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1162" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I1162" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J1162" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1162" t="n">
+        <v>36297695</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1163" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1163" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1163" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I1163" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J1163" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1163" t="n">
+        <v>36298057</v>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1164" t="n">
+        <v>19</v>
+      </c>
+      <c r="G1164" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1164" t="inlineStr">
+        <is>
+          <t>19/36</t>
+        </is>
+      </c>
+      <c r="I1164" s="5" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="J1164" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1164" t="n">
+        <v>40188453</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1156"/>
+  <autoFilter ref="A1:K1164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-24)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1171</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1164"/>
+  <dimension ref="A1:K1171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55183,8 +55183,337 @@
         <v>40188453</v>
       </c>
     </row>
+    <row r="1165">
+      <c r="A1165" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1165" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1165" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1165" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I1165" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J1165" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1165" t="n">
+        <v>36321420</v>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1166" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1166" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
+      </c>
+      <c r="I1166" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J1166" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1166" t="n">
+        <v>36929302</v>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1167" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1167" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1167" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I1167" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1167" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1167" t="n">
+        <v>36298351</v>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F1168" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1168" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1168" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1168" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1168" t="n">
+        <v>36298392</v>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1169" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1169" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1169" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1169" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1169" t="n">
+        <v>36298589</v>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1170" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1170" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="I1170" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1170" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1170" t="n">
+        <v>40189912</v>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1171" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1171" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>3/24</t>
+        </is>
+      </c>
+      <c r="I1171" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J1171" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1171" t="n">
+        <v>43379246</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1164"/>
+  <autoFilter ref="A1:K1171"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-25)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1171"/>
+  <dimension ref="A1:K1185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55512,8 +55512,666 @@
         <v>43379246</v>
       </c>
     </row>
+    <row r="1172">
+      <c r="A1172" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1172" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1172" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1172" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1172" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1172" t="n">
+        <v>37090016</v>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1173" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1173" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>5/7</t>
+        </is>
+      </c>
+      <c r="I1173" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J1173" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1173" t="n">
+        <v>42435331</v>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1174" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1174" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1174" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1174" t="n">
+        <v>42435131</v>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1175" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1175" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1175" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1175" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1175" t="n">
+        <v>37230124</v>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1176" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1176" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1176" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1176" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1176" t="n">
+        <v>37230160</v>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1177" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1177" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1177" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1177" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1177" t="n">
+        <v>37090974</v>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1178" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1178" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1178" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1178" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1178" t="n">
+        <v>42430591</v>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1179" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1179" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>3/7</t>
+        </is>
+      </c>
+      <c r="I1179" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J1179" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1179" t="n">
+        <v>42431394</v>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1180" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1180" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1180" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1180" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1180" t="n">
+        <v>36321571</v>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1181" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1181" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>2/18</t>
+        </is>
+      </c>
+      <c r="I1181" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J1181" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1181" t="n">
+        <v>36929393</v>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1182" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1182" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I1182" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1182" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1182" t="n">
+        <v>36298766</v>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1183" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1183" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1183" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1183" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1183" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I1183" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1183" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1183" t="n">
+        <v>36298820</v>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1184" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1184" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1184" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1184" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1184" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I1184" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1184" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1184" t="n">
+        <v>36298873</v>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1185" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1185" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1185" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1185" t="n">
+        <v>11</v>
+      </c>
+      <c r="H1185" t="inlineStr">
+        <is>
+          <t>10/11</t>
+        </is>
+      </c>
+      <c r="I1185" s="3" t="n">
+        <v>90.90000000000001</v>
+      </c>
+      <c r="J1185" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1185" t="n">
+        <v>40190140</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1171"/>
+  <autoFilter ref="A1:K1185"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-26)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1185"/>
+  <dimension ref="A1:K1192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56170,8 +56170,337 @@
         <v>40190140</v>
       </c>
     </row>
+    <row r="1186">
+      <c r="A1186" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1186" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1186" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1186" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1186" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1186" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I1186" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J1186" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1186" t="n">
+        <v>36319509</v>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1187" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1187" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1187" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1187" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1187" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I1187" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1187" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1187" t="n">
+        <v>36320066</v>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D1188" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1188" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1188" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1188" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1188" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I1188" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1188" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1188" t="n">
+        <v>36320667</v>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1189" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1189" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F1189" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1189" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1189" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1189" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1189" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1189" t="n">
+        <v>36320790</v>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D1190" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1190" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1190" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1190" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1190" t="inlineStr">
+        <is>
+          <t>22/28</t>
+        </is>
+      </c>
+      <c r="I1190" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J1190" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1190" t="n">
+        <v>36320900</v>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D1191" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1191" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1191" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1191" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1191" t="inlineStr">
+        <is>
+          <t>21/36</t>
+        </is>
+      </c>
+      <c r="I1191" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J1191" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1191" t="n">
+        <v>36893837</v>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1192" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1192" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1192" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1192" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1192" t="inlineStr">
+        <is>
+          <t>8/36</t>
+        </is>
+      </c>
+      <c r="I1192" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1192" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1192" t="n">
+        <v>36893905</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1185"/>
+  <autoFilter ref="A1:K1192"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-27)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1192"/>
+  <dimension ref="A1:K1200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56499,8 +56499,384 @@
         <v>36893905</v>
       </c>
     </row>
+    <row r="1193">
+      <c r="A1193" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1193" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1193" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1193" t="n">
+        <v>32</v>
+      </c>
+      <c r="H1193" t="inlineStr">
+        <is>
+          <t>4/32</t>
+        </is>
+      </c>
+      <c r="I1193" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J1193" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1193" t="n">
+        <v>43470836</v>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>Guided Session (English version)</t>
+        </is>
+      </c>
+      <c r="E1194" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1194" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1194" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1194" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1194" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1194" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1194" t="n">
+        <v>36323130</v>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1195" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1195" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1195" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1195" t="inlineStr">
+        <is>
+          <t>9/36</t>
+        </is>
+      </c>
+      <c r="I1195" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1195" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1195" t="n">
+        <v>38771782</v>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1196" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1196" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1196" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1196" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I1196" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J1196" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1196" t="n">
+        <v>36329212</v>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1197" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1197" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1197" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1197" t="inlineStr">
+        <is>
+          <t>20/36</t>
+        </is>
+      </c>
+      <c r="I1197" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J1197" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1197" t="n">
+        <v>38771882</v>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1198" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1198" t="n">
+        <v>36</v>
+      </c>
+      <c r="G1198" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1198" t="inlineStr">
+        <is>
+          <t>36/28</t>
+        </is>
+      </c>
+      <c r="I1198" s="3" t="n">
+        <v>128.6</v>
+      </c>
+      <c r="J1198" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1198" t="n">
+        <v>36329977</v>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1199" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1199" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1199" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1199" t="inlineStr">
+        <is>
+          <t>16/36</t>
+        </is>
+      </c>
+      <c r="I1199" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1199" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1199" t="n">
+        <v>36323869</v>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1200" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1200" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1200" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1200" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1200" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1200" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1200" t="n">
+        <v>36935884</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1192"/>
+  <autoFilter ref="A1:K1200"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-28)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1208</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1200"/>
+  <dimension ref="A1:K1208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56875,8 +56875,384 @@
         <v>36935884</v>
       </c>
     </row>
+    <row r="1201">
+      <c r="A1201" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1201" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1201" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1201" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1201" t="inlineStr">
+        <is>
+          <t>4/36</t>
+        </is>
+      </c>
+      <c r="I1201" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J1201" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1201" t="n">
+        <v>37240294</v>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1202" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1202" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1202" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1202" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1202" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1202" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1202" t="n">
+        <v>36336040</v>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1203" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1203" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1203" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1203" t="inlineStr">
+        <is>
+          <t>12/36</t>
+        </is>
+      </c>
+      <c r="I1203" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1203" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1203" t="n">
+        <v>37240437</v>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1204" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1204" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1204" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1204" t="inlineStr">
+        <is>
+          <t>21/36</t>
+        </is>
+      </c>
+      <c r="I1204" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J1204" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1204" t="n">
+        <v>36892154</v>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1205" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1205" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1205" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1205" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1205" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1205" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1205" t="n">
+        <v>36336255</v>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1206" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1206" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1206" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1206" t="inlineStr">
+        <is>
+          <t>26/28</t>
+        </is>
+      </c>
+      <c r="I1206" s="3" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="J1206" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1206" t="n">
+        <v>36692767</v>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1207" t="n">
+        <v>37</v>
+      </c>
+      <c r="G1207" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1207" t="inlineStr">
+        <is>
+          <t>37/36</t>
+        </is>
+      </c>
+      <c r="I1207" s="3" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="J1207" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1207" t="n">
+        <v>42481095</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1208" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1208" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1208" t="inlineStr">
+        <is>
+          <t>31/36</t>
+        </is>
+      </c>
+      <c r="I1208" s="3" t="n">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="J1208" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1208" t="n">
+        <v>36892109</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1200"/>
+  <autoFilter ref="A1:K1208"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-29)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1216</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1208"/>
+  <dimension ref="A1:K1216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57251,8 +57251,384 @@
         <v>36892109</v>
       </c>
     </row>
+    <row r="1209">
+      <c r="A1209" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1209" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1209" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1209" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I1209" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1209" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1209" t="n">
+        <v>36390341</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1210" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1210" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I1210" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J1210" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1210" t="n">
+        <v>36281144</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1211" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1211" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I1211" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1211" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1211" t="n">
+        <v>38531920</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1212" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1212" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>15/18</t>
+        </is>
+      </c>
+      <c r="I1212" s="5" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="J1212" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1212" t="n">
+        <v>36928739</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1213" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1213" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I1213" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J1213" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1213" t="n">
+        <v>36281008</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1214" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1214" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1214" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1214" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1214" t="n">
+        <v>37873150</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1215" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1215" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1215" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1215" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1215" t="n">
+        <v>36929045</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1216" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1216" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>11/24</t>
+        </is>
+      </c>
+      <c r="I1216" s="4" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="J1216" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1216" t="n">
+        <v>43379248</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1208"/>
+  <autoFilter ref="A1:K1216"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-30)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1224</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1216"/>
+  <dimension ref="A1:K1224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57627,8 +57627,384 @@
         <v>43379248</v>
       </c>
     </row>
+    <row r="1217">
+      <c r="A1217" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1217" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1217" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1217" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I1217" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J1217" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1217" t="n">
+        <v>36321372</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1218" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1218" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1218" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1218" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1218" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1218" t="n">
+        <v>40188424</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1219" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1219" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1219" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I1219" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1219" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1219" t="n">
+        <v>36929171</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1220" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1220" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>3/18</t>
+        </is>
+      </c>
+      <c r="I1220" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1220" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1220" t="n">
+        <v>36298251</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F1221" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1221" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I1221" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J1221" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1221" t="n">
+        <v>36297696</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1222" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1222" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1222" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1222" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1222" t="n">
+        <v>36298058</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1223" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1223" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1223" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1223" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1223" t="n">
+        <v>40188454</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1224" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1224" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1224" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>14/24</t>
+        </is>
+      </c>
+      <c r="I1224" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J1224" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1224" t="n">
+        <v>43379249</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1216"/>
+  <autoFilter ref="A1:K1224"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-01)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1224</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1231</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1224"/>
+  <dimension ref="A1:K1231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57558,22 +57558,22 @@
         </is>
       </c>
       <c r="F1215" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G1215" t="n">
         <v>8</v>
       </c>
       <c r="H1215" t="inlineStr">
         <is>
-          <t>8/8</t>
+          <t>7/8</t>
         </is>
       </c>
       <c r="I1215" s="3" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="J1215" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="K1215" t="n">
@@ -58003,8 +58003,337 @@
         <v>43379249</v>
       </c>
     </row>
+    <row r="1225">
+      <c r="A1225" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1225" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1225" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1225" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I1225" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J1225" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1225" t="n">
+        <v>36321421</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1226" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1226" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1226" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I1226" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J1226" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1226" t="n">
+        <v>36929303</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1227" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1227" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1227" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I1227" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1227" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1227" t="n">
+        <v>36298352</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1228" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F1228" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1228" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>26/28</t>
+        </is>
+      </c>
+      <c r="I1228" s="3" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="J1228" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1228" t="n">
+        <v>36298393</v>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1229" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1229" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1229" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1229" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1229" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1229" t="n">
+        <v>36298590</v>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1230" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1230" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1230" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1230" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1230" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1230" t="n">
+        <v>40189914</v>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1231" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1231" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1231" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>10/24</t>
+        </is>
+      </c>
+      <c r="I1231" s="4" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="J1231" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1231" t="n">
+        <v>43379250</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1224"/>
+  <autoFilter ref="A1:K1231"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-02)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1231</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1245</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1231"/>
+  <dimension ref="A1:K1245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57934,22 +57934,22 @@
         </is>
       </c>
       <c r="F1223" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G1223" t="n">
         <v>8</v>
       </c>
       <c r="H1223" t="inlineStr">
         <is>
-          <t>8/8</t>
+          <t>7/8</t>
         </is>
       </c>
       <c r="I1223" s="3" t="n">
-        <v>100</v>
+        <v>87.5</v>
       </c>
       <c r="J1223" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="K1223" t="n">
@@ -58332,8 +58332,666 @@
         <v>43379250</v>
       </c>
     </row>
+    <row r="1232">
+      <c r="A1232" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1232" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1232" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1232" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>2/28</t>
+        </is>
+      </c>
+      <c r="I1232" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="J1232" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1232" t="n">
+        <v>37090017</v>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1233" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1233" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1233" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1233" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1233" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1233" t="n">
+        <v>42435132</v>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1234" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1234" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1234" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1234" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1234" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1234" t="n">
+        <v>37230125</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1235" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1235" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1235" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1235" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1235" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1235" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1235" t="n">
+        <v>37230161</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1236" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1236" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1236" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>3/7</t>
+        </is>
+      </c>
+      <c r="I1236" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J1236" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1236" t="n">
+        <v>37090975</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1237" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1237" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1237" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1237" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1237" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1237" t="n">
+        <v>42430592</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1238" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1238" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1238" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>4/7</t>
+        </is>
+      </c>
+      <c r="I1238" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J1238" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1238" t="n">
+        <v>42431395</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1239" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1239" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1239" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I1239" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J1239" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1239" t="n">
+        <v>36321572</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1240" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1240" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1240" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I1240" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1240" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1240" t="n">
+        <v>36929394</v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1241" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1241" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1241" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I1241" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1241" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1241" t="n">
+        <v>36298767</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1242" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1242" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1242" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1242" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1242" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1242" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1242" t="n">
+        <v>36298821</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1243" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1243" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1243" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1243" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1243" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1243" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1243" t="n">
+        <v>36298874</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1244" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1244" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1244" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1244" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1244" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1244" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1244" t="n">
+        <v>40190141</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1245" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1245" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1245" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1245" t="inlineStr">
+        <is>
+          <t>7/24</t>
+        </is>
+      </c>
+      <c r="I1245" s="4" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="J1245" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1245" t="n">
+        <v>43379251</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1231"/>
+  <autoFilter ref="A1:K1245"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-03)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1245</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1257</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1245"/>
+  <dimension ref="A1:K1257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58990,8 +58990,572 @@
         <v>43379251</v>
       </c>
     </row>
+    <row r="1246">
+      <c r="A1246" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1246" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1246" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1246" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1246" t="inlineStr">
+        <is>
+          <t>10/34</t>
+        </is>
+      </c>
+      <c r="I1246" s="4" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="J1246" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1246" t="n">
+        <v>36319510</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1247" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1247" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1247" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1247" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1247" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1247" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1247" t="n">
+        <v>36320067</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1248" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1248" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1248" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1248" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1248" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1248" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1248" t="n">
+        <v>36320668</v>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1249" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1249" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1249" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1249" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="I1249" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J1249" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1249" t="n">
+        <v>43355389</v>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1250" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1250" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1250" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1250" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1250" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1250" t="n">
+        <v>43355513</v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1251" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1251" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1251" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1251" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1251" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1251" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1251" t="n">
+        <v>43355770</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1252" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1252" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1252" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1252" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1252" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1252" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1252" t="n">
+        <v>43355901</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1253" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1253" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1253" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1253" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1253" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1253" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1253" t="n">
+        <v>43355903</v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1254" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1254" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1254" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1254" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="I1254" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1254" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1254" t="n">
+        <v>43355911</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1255" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1255" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1255" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1255" t="inlineStr">
+        <is>
+          <t>29/28</t>
+        </is>
+      </c>
+      <c r="I1255" s="3" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="J1255" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1255" t="n">
+        <v>36320901</v>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1256" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1256" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1256" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1256" t="inlineStr">
+        <is>
+          <t>29/36</t>
+        </is>
+      </c>
+      <c r="I1256" s="5" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="J1256" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1256" t="n">
+        <v>36893838</v>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1257" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1257" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1257" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1257" t="inlineStr">
+        <is>
+          <t>4/36</t>
+        </is>
+      </c>
+      <c r="I1257" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J1257" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1257" t="n">
+        <v>36893908</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1245"/>
+  <autoFilter ref="A1:K1257"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-04)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1257</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1265</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1257"/>
+  <dimension ref="A1:K1265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -59554,8 +59554,384 @@
         <v>36893908</v>
       </c>
     </row>
+    <row r="1258">
+      <c r="A1258" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1258" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1258" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1258" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1258" t="inlineStr">
+        <is>
+          <t>5/36</t>
+        </is>
+      </c>
+      <c r="I1258" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="J1258" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1258" t="n">
+        <v>36323285</v>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1259" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1259" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1259" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1259" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I1259" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J1259" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1259" t="n">
+        <v>36323131</v>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1260" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1260" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1260" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1260" t="inlineStr">
+        <is>
+          <t>8/36</t>
+        </is>
+      </c>
+      <c r="I1260" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1260" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1260" t="n">
+        <v>38771783</v>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1261" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1261" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1261" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1261" t="inlineStr">
+        <is>
+          <t>12/28</t>
+        </is>
+      </c>
+      <c r="I1261" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J1261" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1261" t="n">
+        <v>36329213</v>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1262" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1262" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1262" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1262" t="inlineStr">
+        <is>
+          <t>16/36</t>
+        </is>
+      </c>
+      <c r="I1262" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1262" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1262" t="n">
+        <v>38771883</v>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1263" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1263" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1263" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1263" t="inlineStr">
+        <is>
+          <t>30/28</t>
+        </is>
+      </c>
+      <c r="I1263" s="3" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="J1263" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1263" t="n">
+        <v>36329978</v>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1264" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1264" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1264" t="inlineStr">
+        <is>
+          <t>17/36</t>
+        </is>
+      </c>
+      <c r="I1264" s="4" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="J1264" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1264" t="n">
+        <v>36323870</v>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1265" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1265" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1265" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1265" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1265" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1265" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1265" t="n">
+        <v>36935885</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1257"/>
+  <autoFilter ref="A1:K1265"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-05)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1265</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1273</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1265"/>
+  <dimension ref="A1:K1273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -59930,8 +59930,384 @@
         <v>36935885</v>
       </c>
     </row>
+    <row r="1266">
+      <c r="A1266" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1266" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1266" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1266" t="inlineStr">
+        <is>
+          <t>13/36</t>
+        </is>
+      </c>
+      <c r="I1266" s="4" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="J1266" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1266" t="n">
+        <v>37240295</v>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1267" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1267" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1267" t="inlineStr">
+        <is>
+          <t>17/28</t>
+        </is>
+      </c>
+      <c r="I1267" s="5" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="J1267" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1267" t="n">
+        <v>36336041</v>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1268" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1268" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1268" t="inlineStr">
+        <is>
+          <t>14/36</t>
+        </is>
+      </c>
+      <c r="I1268" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1268" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1268" t="n">
+        <v>37240438</v>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1269" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1269" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1269" t="inlineStr">
+        <is>
+          <t>23/36</t>
+        </is>
+      </c>
+      <c r="I1269" s="5" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="J1269" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1269" t="n">
+        <v>36892155</v>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1270" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1270" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1270" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1270" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1270" t="n">
+        <v>36336256</v>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1271" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1271" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1271" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1271" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1271" t="n">
+        <v>36692768</v>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1272" t="n">
+        <v>36</v>
+      </c>
+      <c r="G1272" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>36/36</t>
+        </is>
+      </c>
+      <c r="I1272" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1272" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1272" t="n">
+        <v>42481096</v>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1273" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1273" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>25/36</t>
+        </is>
+      </c>
+      <c r="I1273" s="5" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="J1273" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1273" t="n">
+        <v>36892110</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1265"/>
+  <autoFilter ref="A1:K1273"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-06)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1273</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1280</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1273"/>
+  <dimension ref="A1:K1280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -60306,8 +60306,337 @@
         <v>36892110</v>
       </c>
     </row>
+    <row r="1274">
+      <c r="A1274" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1274" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1274" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I1274" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J1274" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1274" t="n">
+        <v>36390342</v>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1275" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1275" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I1275" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J1275" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1275" t="n">
+        <v>36281145</v>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1276" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1276" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I1276" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1276" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1276" t="n">
+        <v>38531921</v>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1277" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1277" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I1277" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1277" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1277" t="n">
+        <v>36928740</v>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1278" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1278" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1278" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1278" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1278" t="n">
+        <v>36281009</v>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1279" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1279" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>26/28</t>
+        </is>
+      </c>
+      <c r="I1279" s="3" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="J1279" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1279" t="n">
+        <v>37873151</v>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1280" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1280" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>8/34</t>
+        </is>
+      </c>
+      <c r="I1280" s="4" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="J1280" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1280" t="n">
+        <v>43379252</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1273"/>
+  <autoFilter ref="A1:K1280"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-07)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1280</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1287</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1280"/>
+  <dimension ref="A1:K1287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -60635,8 +60635,337 @@
         <v>43379252</v>
       </c>
     </row>
+    <row r="1281">
+      <c r="A1281" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1281" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1281" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I1281" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J1281" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1281" t="n">
+        <v>36321373</v>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1282" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1282" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1282" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1282" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1282" t="n">
+        <v>40188425</v>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1283" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1283" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I1283" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1283" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1283" t="n">
+        <v>36929172</v>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1284" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1284" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I1284" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1284" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1284" t="n">
+        <v>36298252</v>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F1285" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1285" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I1285" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J1285" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1285" t="n">
+        <v>36297697</v>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1286" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1286" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1286" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1286" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1286" t="n">
+        <v>36298059</v>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1287" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1287" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>15/34</t>
+        </is>
+      </c>
+      <c r="I1287" s="4" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="J1287" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1287" t="n">
+        <v>43379253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1280"/>
+  <autoFilter ref="A1:K1287"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-08)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1287</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1294</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1287"/>
+  <dimension ref="A1:K1294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -60964,8 +60964,337 @@
         <v>43379253</v>
       </c>
     </row>
+    <row r="1288">
+      <c r="A1288" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1288" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1288" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I1288" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1288" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1288" t="n">
+        <v>36321422</v>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1289" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1289" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
+      </c>
+      <c r="I1289" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J1289" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1289" t="n">
+        <v>36929304</v>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1290" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1290" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I1290" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1290" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1290" t="n">
+        <v>36298353</v>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F1291" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1291" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1291" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1291" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1291" t="n">
+        <v>36298394</v>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1292" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1292" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1292" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1292" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1292" t="n">
+        <v>36298591</v>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1293" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1293" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="I1293" s="3" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="J1293" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1293" t="n">
+        <v>40189916</v>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1294" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1294" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>14/34</t>
+        </is>
+      </c>
+      <c r="I1294" s="4" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="J1294" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1294" t="n">
+        <v>43379254</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1287"/>
+  <autoFilter ref="A1:K1294"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-09)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1307</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1294"/>
+  <dimension ref="A1:K1307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -61293,8 +61293,619 @@
         <v>43379254</v>
       </c>
     </row>
+    <row r="1295">
+      <c r="A1295" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1295" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1295" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="I1295" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1295" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1295" t="n">
+        <v>37090018</v>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1296" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1296" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1296" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1296" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1296" t="n">
+        <v>42435133</v>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1297" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1297" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1297" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1297" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1297" t="n">
+        <v>37230126</v>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1298" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1298" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1298" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1298" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1298" t="n">
+        <v>37230162</v>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1299" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1299" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1299" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1299" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1299" t="n">
+        <v>37090976</v>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1300" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1300" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>3/7</t>
+        </is>
+      </c>
+      <c r="I1300" s="4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="J1300" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1300" t="n">
+        <v>42430593</v>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1301" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1301" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1301" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1301" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1301" t="n">
+        <v>42431396</v>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1302" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1302" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I1302" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J1302" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1302" t="n">
+        <v>36321573</v>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1303" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1303" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I1303" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1303" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1303" t="n">
+        <v>36929395</v>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1304" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1304" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I1304" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1304" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1304" t="n">
+        <v>36298768</v>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1305" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1305" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1305" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1305" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1305" t="n">
+        <v>36298822</v>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1306" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1306" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>22/28</t>
+        </is>
+      </c>
+      <c r="I1306" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J1306" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1306" t="n">
+        <v>36298875</v>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1307" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1307" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>17/34</t>
+        </is>
+      </c>
+      <c r="I1307" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1307" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1307" t="n">
+        <v>43379255</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1294"/>
+  <autoFilter ref="A1:K1307"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-10)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1307</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1320</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1307"/>
+  <dimension ref="A1:K1320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -61904,8 +61904,619 @@
         <v>43379255</v>
       </c>
     </row>
+    <row r="1308">
+      <c r="A1308" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1308" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1308" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I1308" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J1308" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1308" t="n">
+        <v>36319511</v>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1309" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1309" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>6/10</t>
+        </is>
+      </c>
+      <c r="I1309" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="J1309" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1309" t="n">
+        <v>42666075</v>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1310" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1310" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1310" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1310" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1310" t="n">
+        <v>36320068</v>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1311" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1311" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1311" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1311" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1311" t="n">
+        <v>36320669</v>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1312" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1312" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="I1312" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J1312" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1312" t="n">
+        <v>43578626</v>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1313" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1313" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1313" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1313" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1313" t="n">
+        <v>43355514</v>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1314" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1314" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1314" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1314" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1314" t="n">
+        <v>43578013</v>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1315" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1315" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1315" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1315" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1315" t="n">
+        <v>43578369</v>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1316" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1316" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1316" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1316" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1316" t="n">
+        <v>43578505</v>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1317" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1317" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="I1317" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1317" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1317" t="n">
+        <v>43578557</v>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1318" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1318" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1318" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1318" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1318" t="n">
+        <v>36320902</v>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1319" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1319" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>15/36</t>
+        </is>
+      </c>
+      <c r="I1319" s="4" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="J1319" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1319" t="n">
+        <v>36893839</v>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1320" t="n">
+        <v>36</v>
+      </c>
+      <c r="G1320" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>36/36</t>
+        </is>
+      </c>
+      <c r="I1320" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1320" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1320" t="n">
+        <v>36893910</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1307"/>
+  <autoFilter ref="A1:K1320"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-11)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1320</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1328</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1320"/>
+  <dimension ref="A1:K1328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58968,18 +58968,18 @@
         </is>
       </c>
       <c r="F1245" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G1245" t="n">
         <v>24</v>
       </c>
       <c r="H1245" t="inlineStr">
         <is>
-          <t>7/24</t>
+          <t>6/24</t>
         </is>
       </c>
       <c r="I1245" s="4" t="n">
-        <v>29.2</v>
+        <v>25</v>
       </c>
       <c r="J1245" t="inlineStr">
         <is>
@@ -62515,8 +62515,384 @@
         <v>36893910</v>
       </c>
     </row>
+    <row r="1321">
+      <c r="A1321" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1321" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1321" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>14/36</t>
+        </is>
+      </c>
+      <c r="I1321" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1321" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1321" t="n">
+        <v>36323286</v>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>Guided Session (English version)</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1322" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1322" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>17/28</t>
+        </is>
+      </c>
+      <c r="I1322" s="5" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="J1322" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1322" t="n">
+        <v>36323132</v>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1323" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1323" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>7/36</t>
+        </is>
+      </c>
+      <c r="I1323" s="4" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="J1323" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1323" t="n">
+        <v>38771784</v>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1324" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1324" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>20/28</t>
+        </is>
+      </c>
+      <c r="I1324" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J1324" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1324" t="n">
+        <v>36329214</v>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1325" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1325" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>21/36</t>
+        </is>
+      </c>
+      <c r="I1325" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J1325" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1325" t="n">
+        <v>38771884</v>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1326" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1326" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>24/28</t>
+        </is>
+      </c>
+      <c r="I1326" s="3" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="J1326" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1326" t="n">
+        <v>36329979</v>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1327" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1327" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>20/36</t>
+        </is>
+      </c>
+      <c r="I1327" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J1327" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1327" t="n">
+        <v>36323871</v>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1328" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1328" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>12/36</t>
+        </is>
+      </c>
+      <c r="I1328" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1328" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1328" t="n">
+        <v>36935886</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1320"/>
+  <autoFilter ref="A1:K1328"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-12)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1328</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1336</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1328"/>
+  <dimension ref="A1:K1336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -62891,8 +62891,384 @@
         <v>36935886</v>
       </c>
     </row>
+    <row r="1329">
+      <c r="A1329" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1329" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1329" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>7/36</t>
+        </is>
+      </c>
+      <c r="I1329" s="4" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="J1329" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1329" t="n">
+        <v>37240296</v>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1330" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1330" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I1330" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J1330" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1330" t="n">
+        <v>36336042</v>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1331" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1331" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>15/36</t>
+        </is>
+      </c>
+      <c r="I1331" s="4" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="J1331" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1331" t="n">
+        <v>37240439</v>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1332" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1332" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>28/36</t>
+        </is>
+      </c>
+      <c r="I1332" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J1332" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1332" t="n">
+        <v>36892156</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1333" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1333" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>30/28</t>
+        </is>
+      </c>
+      <c r="I1333" s="3" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="J1333" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1333" t="n">
+        <v>36336257</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1334" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1334" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1334" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1334" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1334" t="n">
+        <v>36692769</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1335" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1335" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>38/36</t>
+        </is>
+      </c>
+      <c r="I1335" s="3" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="J1335" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1335" t="n">
+        <v>42481097</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1336" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1336" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>15/36</t>
+        </is>
+      </c>
+      <c r="I1336" s="4" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="J1336" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1336" t="n">
+        <v>36892111</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1328"/>
+  <autoFilter ref="A1:K1336"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-13)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1336</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1348</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1336"/>
+  <dimension ref="A1:K1348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63267,8 +63267,572 @@
         <v>36892111</v>
       </c>
     </row>
+    <row r="1337">
+      <c r="A1337" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1337" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1337" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1337" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1337" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1337" t="n">
+        <v>43815253</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1338" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1338" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1338" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1338" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1338" t="n">
+        <v>43815368</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1339" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1339" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1339" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1339" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1339" t="n">
+        <v>43815393</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1340" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1340" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1340" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1340" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1340" t="n">
+        <v>43815418</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1341" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1341" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1341" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I1341" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J1341" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1341" t="n">
+        <v>36390343</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1342" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1342" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1342" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I1342" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1342" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1342" t="n">
+        <v>36281146</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1343" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1343" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1343" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I1343" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1343" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1343" t="n">
+        <v>38531922</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1344" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1344" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1344" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="I1344" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J1344" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1344" t="n">
+        <v>36928741</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1345" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1345" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1345" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1345" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1345" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1345" t="n">
+        <v>36281010</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1346" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1346" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1346" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1346" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1346" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1346" t="n">
+        <v>37873152</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1347" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1347" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1347" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1347" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1347" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1347" t="n">
+        <v>36929047</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1348" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1348" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1348" t="inlineStr">
+        <is>
+          <t>10/34</t>
+        </is>
+      </c>
+      <c r="I1348" s="4" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="J1348" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1348" t="n">
+        <v>43379256</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1336"/>
+  <autoFilter ref="A1:K1348"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-16)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1348</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1370</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1348"/>
+  <dimension ref="A1:K1370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -63668,18 +63668,18 @@
         </is>
       </c>
       <c r="F1345" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G1345" t="n">
         <v>28</v>
       </c>
       <c r="H1345" t="inlineStr">
         <is>
-          <t>23/28</t>
+          <t>22/28</t>
         </is>
       </c>
       <c r="I1345" s="5" t="n">
-        <v>82.09999999999999</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="J1345" t="inlineStr">
         <is>
@@ -63831,8 +63831,1042 @@
         <v>43379256</v>
       </c>
     </row>
+    <row r="1349">
+      <c r="A1349" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1349" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1349" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1349" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I1349" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J1349" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1349" t="n">
+        <v>36321374</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1350" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1350" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1350" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1350" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1350" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1350" t="n">
+        <v>40188426</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1351" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1351" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1351" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I1351" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1351" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1351" t="n">
+        <v>36929173</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1352" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1352" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1352" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I1352" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1352" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1352" t="n">
+        <v>36298253</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F1353" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1353" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1353" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I1353" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1353" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1353" t="n">
+        <v>36297698</v>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1354" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1354" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I1354" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J1354" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1354" t="n">
+        <v>36298060</v>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1355" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1355" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1355" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1355" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1355" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1355" t="n">
+        <v>40188456</v>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1356" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1356" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1356" t="inlineStr">
+        <is>
+          <t>7/34</t>
+        </is>
+      </c>
+      <c r="I1356" s="4" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="J1356" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1356" t="n">
+        <v>43379257</v>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1357" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1357" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1357" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I1357" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J1357" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1357" t="n">
+        <v>36321423</v>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1358" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1358" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1358" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I1358" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1358" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1358" t="n">
+        <v>36929305</v>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1359" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1359" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1359" t="inlineStr">
+        <is>
+          <t>18/18</t>
+        </is>
+      </c>
+      <c r="I1359" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1359" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1359" t="n">
+        <v>36298354</v>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F1360" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1360" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1360" t="inlineStr">
+        <is>
+          <t>29/28</t>
+        </is>
+      </c>
+      <c r="I1360" s="3" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="J1360" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1360" t="n">
+        <v>36298395</v>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1361" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1361" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1361" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I1361" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1361" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1361" t="n">
+        <v>36298592</v>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1362" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1362" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1362" t="inlineStr">
+        <is>
+          <t>0/8</t>
+        </is>
+      </c>
+      <c r="I1362" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1362" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1362" t="n">
+        <v>40189917</v>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1363" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1363" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1363" t="inlineStr">
+        <is>
+          <t>0/24</t>
+        </is>
+      </c>
+      <c r="I1363" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1363" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1363" t="n">
+        <v>43379258</v>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1364" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1364" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1364" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I1364" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J1364" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1364" t="n">
+        <v>36321574</v>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1365" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1365" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1365" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I1365" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J1365" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1365" t="n">
+        <v>36929396</v>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1366" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1366" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1366" t="inlineStr">
+        <is>
+          <t>13/18</t>
+        </is>
+      </c>
+      <c r="I1366" s="5" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="J1366" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1366" t="n">
+        <v>36298769</v>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1367" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1367" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1367" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I1367" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J1367" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1367" t="n">
+        <v>36298823</v>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1368" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1368" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1368" t="inlineStr">
+        <is>
+          <t>31/28</t>
+        </is>
+      </c>
+      <c r="I1368" s="3" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="J1368" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1368" t="n">
+        <v>36298876</v>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1369" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1369" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1369" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="I1369" s="3" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="J1369" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1369" t="n">
+        <v>40190143</v>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1370" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1370" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1370" t="inlineStr">
+        <is>
+          <t>18/34</t>
+        </is>
+      </c>
+      <c r="I1370" s="5" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="J1370" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1370" t="n">
+        <v>43379259</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1348"/>
+  <autoFilter ref="A1:K1370"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-17)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1370</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1387</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1370"/>
+  <dimension ref="A1:K1387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64865,8 +64865,807 @@
         <v>43379259</v>
       </c>
     </row>
+    <row r="1371">
+      <c r="A1371" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1371" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1371" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1371" t="inlineStr">
+        <is>
+          <t>1/28</t>
+        </is>
+      </c>
+      <c r="I1371" s="4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J1371" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1371" t="n">
+        <v>43815504</v>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1372" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1372" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1372" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1372" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1372" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1372" t="n">
+        <v>43815546</v>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1373" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1373" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1373" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1373" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1373" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1373" t="n">
+        <v>43815643</v>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1374" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1374" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1374" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1374" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1374" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1374" t="n">
+        <v>43815667</v>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1375" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1375" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1375" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1375" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1375" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1375" t="n">
+        <v>43816187</v>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1376" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1376" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1376" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1376" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1376" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1376" t="n">
+        <v>43816532</v>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1377" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1377" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1377" t="inlineStr">
+        <is>
+          <t>1/28</t>
+        </is>
+      </c>
+      <c r="I1377" s="4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J1377" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1377" t="n">
+        <v>36319512</v>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1378" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1378" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1378" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1378" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1378" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1378" t="n">
+        <v>44112615</v>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1379" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1379" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="I1379" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1379" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1379" t="n">
+        <v>36320069</v>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1380" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1380" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1380" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1380" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1380" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1380" t="n">
+        <v>36320670</v>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1381" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1381" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1381" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1381" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1381" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1381" t="n">
+        <v>43355515</v>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1382" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1382" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1382" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1382" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1382" t="n">
+        <v>43578014</v>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1383" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1383" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1383" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1383" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1383" t="n">
+        <v>43816535</v>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1384" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1384" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="I1384" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J1384" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1384" t="n">
+        <v>43578506</v>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1385" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1385" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1385" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1385" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1385" t="n">
+        <v>36320903</v>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1386" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1386" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>16/36</t>
+        </is>
+      </c>
+      <c r="I1386" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1386" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1386" t="n">
+        <v>36893840</v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1387" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1387" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>16/36</t>
+        </is>
+      </c>
+      <c r="I1387" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1387" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1387" t="n">
+        <v>36893913</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1370"/>
+  <autoFilter ref="A1:K1387"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-18)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1387</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1395</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1387"/>
+  <dimension ref="A1:K1395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -65664,8 +65664,384 @@
         <v>36893913</v>
       </c>
     </row>
+    <row r="1388">
+      <c r="A1388" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1388" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1388" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1388" t="inlineStr">
+        <is>
+          <t>13/36</t>
+        </is>
+      </c>
+      <c r="I1388" s="4" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="J1388" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1388" t="n">
+        <v>36323287</v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>Guided Session (English version)</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1389" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1389" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>16/28</t>
+        </is>
+      </c>
+      <c r="I1389" s="5" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="J1389" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1389" t="n">
+        <v>36323133</v>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1390" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1390" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>8/36</t>
+        </is>
+      </c>
+      <c r="I1390" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1390" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1390" t="n">
+        <v>38771785</v>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1391" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1391" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1391" t="inlineStr">
+        <is>
+          <t>14/28</t>
+        </is>
+      </c>
+      <c r="I1391" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1391" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1391" t="n">
+        <v>36329215</v>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1392" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1392" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1392" t="inlineStr">
+        <is>
+          <t>27/36</t>
+        </is>
+      </c>
+      <c r="I1392" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1392" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1392" t="n">
+        <v>38771885</v>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1393" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1393" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1393" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1393" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1393" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1393" t="n">
+        <v>36329980</v>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1394" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1394" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1394" t="inlineStr">
+        <is>
+          <t>12/36</t>
+        </is>
+      </c>
+      <c r="I1394" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1394" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1394" t="n">
+        <v>36323872</v>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1395" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1395" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1395" t="inlineStr">
+        <is>
+          <t>2/36</t>
+        </is>
+      </c>
+      <c r="I1395" s="4" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="J1395" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1395" t="n">
+        <v>36935887</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1387"/>
+  <autoFilter ref="A1:K1395"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-19)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1395</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1403</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1395"/>
+  <dimension ref="A1:K1403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57041,18 +57041,18 @@
         </is>
       </c>
       <c r="F1204" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G1204" t="n">
         <v>36</v>
       </c>
       <c r="H1204" t="inlineStr">
         <is>
-          <t>21/36</t>
+          <t>20/36</t>
         </is>
       </c>
       <c r="I1204" s="5" t="n">
-        <v>58.3</v>
+        <v>55.6</v>
       </c>
       <c r="J1204" t="inlineStr">
         <is>
@@ -66040,8 +66040,384 @@
         <v>36935887</v>
       </c>
     </row>
+    <row r="1396">
+      <c r="A1396" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1396" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1396" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1396" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1396" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1396" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1396" t="n">
+        <v>37240297</v>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1397" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1397" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>22/28</t>
+        </is>
+      </c>
+      <c r="I1397" s="5" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="J1397" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1397" t="n">
+        <v>36336043</v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1398" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1398" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>16/36</t>
+        </is>
+      </c>
+      <c r="I1398" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1398" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1398" t="n">
+        <v>37240440</v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1399" t="n">
+        <v>19</v>
+      </c>
+      <c r="G1399" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>19/36</t>
+        </is>
+      </c>
+      <c r="I1399" s="5" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="J1399" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1399" t="n">
+        <v>36892157</v>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1400" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1400" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1400" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1400" t="inlineStr">
+        <is>
+          <t>31/28</t>
+        </is>
+      </c>
+      <c r="I1400" s="3" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="J1400" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1400" t="n">
+        <v>36336258</v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1401" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1401" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1401" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1401" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1401" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1401" t="n">
+        <v>36692770</v>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1402" t="n">
+        <v>36</v>
+      </c>
+      <c r="G1402" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1402" t="inlineStr">
+        <is>
+          <t>36/36</t>
+        </is>
+      </c>
+      <c r="I1402" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1402" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1402" t="n">
+        <v>42481098</v>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1403" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1403" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1403" t="inlineStr">
+        <is>
+          <t>23/36</t>
+        </is>
+      </c>
+      <c r="I1403" s="5" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="J1403" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1403" t="n">
+        <v>36892112</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1395"/>
+  <autoFilter ref="A1:K1403"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-20)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1403</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1416</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1403"/>
+  <dimension ref="A1:K1416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66416,8 +66416,619 @@
         <v>36892112</v>
       </c>
     </row>
+    <row r="1404">
+      <c r="A1404" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1404" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1404" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1404" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1404" t="inlineStr">
+        <is>
+          <t>2/24</t>
+        </is>
+      </c>
+      <c r="I1404" s="4" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="J1404" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1404" t="n">
+        <v>43815079</v>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1405" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1405" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1405" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1405" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1405" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1405" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1405" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1405" t="n">
+        <v>43815254</v>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1406" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1406" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1406" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1406" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1406" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1406" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1406" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1406" t="n">
+        <v>43815369</v>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1407" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1407" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1407" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1407" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1407" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1407" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1407" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1407" t="n">
+        <v>43815394</v>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1408" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1408" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1408" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1408" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1408" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1408" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1408" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1408" t="n">
+        <v>43815419</v>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1409" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1409" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1409" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1409" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1409" t="inlineStr">
+        <is>
+          <t>4/28</t>
+        </is>
+      </c>
+      <c r="I1409" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1409" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1409" t="n">
+        <v>36390344</v>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1410" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1410" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1410" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1410" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1410" t="inlineStr">
+        <is>
+          <t>2/28</t>
+        </is>
+      </c>
+      <c r="I1410" s="4" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="J1410" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1410" t="n">
+        <v>36281147</v>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1411" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1411" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1411" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1411" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1411" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I1411" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1411" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1411" t="n">
+        <v>38531923</v>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1412" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1412" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1412" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1412" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1412" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I1412" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J1412" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1412" t="n">
+        <v>36928742</v>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1413" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1413" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1413" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1413" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1413" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I1413" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J1413" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1413" t="n">
+        <v>36281011</v>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1414" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1414" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1414" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1414" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1414" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1414" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1414" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1414" t="n">
+        <v>37873153</v>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1415" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1415" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1415" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1415" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1415" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1415" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1415" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1415" t="n">
+        <v>36929048</v>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" s="2" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1416" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1416" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1416" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1416" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1416" t="inlineStr">
+        <is>
+          <t>12/34</t>
+        </is>
+      </c>
+      <c r="I1416" s="4" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="J1416" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1416" t="n">
+        <v>43379260</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1403"/>
+  <autoFilter ref="A1:K1416"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-21)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1416</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1424</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1416"/>
+  <dimension ref="A1:K1424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -67027,8 +67027,384 @@
         <v>43379260</v>
       </c>
     </row>
+    <row r="1417">
+      <c r="A1417" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1417" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1417" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1417" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1417" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1417" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="I1417" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1417" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1417" t="n">
+        <v>36321375</v>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1418" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1418" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1418" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1418" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1418" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1418" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1418" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1418" t="n">
+        <v>40188427</v>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1419" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1419" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1419" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1419" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1419" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I1419" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1419" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1419" t="n">
+        <v>36929174</v>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1420" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1420" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1420" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1420" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1420" t="inlineStr">
+        <is>
+          <t>7/18</t>
+        </is>
+      </c>
+      <c r="I1420" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1420" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1420" t="n">
+        <v>36298254</v>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1421" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1421" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F1421" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1421" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1421" t="inlineStr">
+        <is>
+          <t>29/28</t>
+        </is>
+      </c>
+      <c r="I1421" s="3" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="J1421" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1421" t="n">
+        <v>36297699</v>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1422" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1422" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1422" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1422" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1422" t="inlineStr">
+        <is>
+          <t>24/28</t>
+        </is>
+      </c>
+      <c r="I1422" s="3" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="J1422" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1422" t="n">
+        <v>36298061</v>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1423" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1423" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1423" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1423" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1423" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="I1423" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1423" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1423" t="n">
+        <v>40188457</v>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1424" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1424" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1424" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1424" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1424" t="inlineStr">
+        <is>
+          <t>15/34</t>
+        </is>
+      </c>
+      <c r="I1424" s="4" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="J1424" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1424" t="n">
+        <v>43379261</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1416"/>
+  <autoFilter ref="A1:K1424"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-22)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1424</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1431</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1424"/>
+  <dimension ref="A1:K1431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -67403,8 +67403,337 @@
         <v>43379261</v>
       </c>
     </row>
+    <row r="1425">
+      <c r="A1425" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1425" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1425" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1425" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1425" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1425" t="inlineStr">
+        <is>
+          <t>17/28</t>
+        </is>
+      </c>
+      <c r="I1425" s="5" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="J1425" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1425" t="n">
+        <v>36321424</v>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1426" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1426" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1426" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1426" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1426" t="inlineStr">
+        <is>
+          <t>13/18</t>
+        </is>
+      </c>
+      <c r="I1426" s="5" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="J1426" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1426" t="n">
+        <v>36929306</v>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1427" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1427" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1427" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1427" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1427" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="I1427" s="5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J1427" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1427" t="n">
+        <v>36298355</v>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1428" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1428" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F1428" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1428" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1428" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1428" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1428" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1428" t="n">
+        <v>36298396</v>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1429" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1429" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1429" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1429" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1429" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1429" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1429" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1429" t="n">
+        <v>36298593</v>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1430" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1430" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1430" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1430" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1430" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="I1430" s="3" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="J1430" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1430" t="n">
+        <v>40189919</v>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1431" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1431" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1431" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1431" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1431" t="inlineStr">
+        <is>
+          <t>5/34</t>
+        </is>
+      </c>
+      <c r="I1431" s="4" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="J1431" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1431" t="n">
+        <v>43379262</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1424"/>
+  <autoFilter ref="A1:K1431"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-23)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1431</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1445</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1431"/>
+  <dimension ref="A1:K1445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -67732,8 +67732,666 @@
         <v>43379262</v>
       </c>
     </row>
+    <row r="1432">
+      <c r="A1432" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1432" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1432" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1432" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1432" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1432" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1432" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1432" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1432" t="n">
+        <v>37090020</v>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D1433" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1433" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1433" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1433" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1433" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1433" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1433" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1433" t="n">
+        <v>42435135</v>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1434" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1434" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1434" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1434" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1434" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1434" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1434" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1434" t="n">
+        <v>37230128</v>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1435" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1435" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1435" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1435" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1435" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1435" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1435" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1435" t="n">
+        <v>37230164</v>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1436" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1436" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1436" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1436" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1436" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1436" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1436" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1436" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1436" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1436" t="n">
+        <v>37090978</v>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1437" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1437" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1437" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1437" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1437" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1437" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1437" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1437" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1437" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1437" t="n">
+        <v>42430595</v>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1438" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1438" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1438" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1438" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1438" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1438" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1438" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1438" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1438" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1438" t="n">
+        <v>42431398</v>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1439" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1439" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1439" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1439" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1439" t="inlineStr">
+        <is>
+          <t>11/28</t>
+        </is>
+      </c>
+      <c r="I1439" s="4" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="J1439" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1439" t="n">
+        <v>36321575</v>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1440" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1440" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1440" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1440" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1440" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1440" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1440" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I1440" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1440" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1440" t="n">
+        <v>36929397</v>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1441" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1441" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1441" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1441" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1441" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1441" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1441" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I1441" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1441" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1441" t="n">
+        <v>36298770</v>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1442" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1442" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1442" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1442" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1442" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1442" t="inlineStr">
+        <is>
+          <t>27/28</t>
+        </is>
+      </c>
+      <c r="I1442" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J1442" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1442" t="n">
+        <v>36298824</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1443" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1443" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1443" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1443" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1443" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1443" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I1443" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1443" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1443" t="n">
+        <v>36298877</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1444" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1444" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1444" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1444" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1444" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1444" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1444" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1444" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1444" t="n">
+        <v>40190144</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1445" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1445" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1445" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1445" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1445" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1445" t="inlineStr">
+        <is>
+          <t>5/34</t>
+        </is>
+      </c>
+      <c r="I1445" s="4" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="J1445" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1445" t="n">
+        <v>43379263</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1431"/>
+  <autoFilter ref="A1:K1445"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-24)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1445</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1463</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1445"/>
+  <dimension ref="A1:K1463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -68390,8 +68390,854 @@
         <v>43379263</v>
       </c>
     </row>
+    <row r="1446">
+      <c r="A1446" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1446" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1446" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1446" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1446" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1446" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1446" t="inlineStr">
+        <is>
+          <t>3/24</t>
+        </is>
+      </c>
+      <c r="I1446" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J1446" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1446" t="n">
+        <v>43815505</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1447" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1447" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1447" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1447" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1447" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1447" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1447" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1447" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1447" t="n">
+        <v>43815547</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1448" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1448" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1448" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1448" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1448" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1448" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1448" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1448" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1448" t="n">
+        <v>43815644</v>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1449" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1449" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1449" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1449" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1449" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1449" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1449" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1449" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1449" t="n">
+        <v>43815668</v>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1450" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1450" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1450" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1450" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1450" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1450" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1450" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1450" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1450" t="n">
+        <v>43816188</v>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1451" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1451" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1451" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1451" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1451" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1451" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1451" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1451" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1451" t="n">
+        <v>44371083</v>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1452" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1452" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1452" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F1452" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1452" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1452" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1452" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1452" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1452" t="n">
+        <v>36319513</v>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1453" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1453" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1453" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1453" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1453" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1453" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+      <c r="I1453" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J1453" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1453" t="n">
+        <v>36320070</v>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1454" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D1454" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1454" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1454" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1454" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1454" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1454" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1454" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1454" t="n">
+        <v>36320671</v>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1455" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D1455" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1455" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1455" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1455" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1455" t="inlineStr">
+        <is>
+          <t>1/8</t>
+        </is>
+      </c>
+      <c r="I1455" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J1455" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1455" t="n">
+        <v>44345196</v>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1456" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D1456" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1456" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1456" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1456" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1456" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1456" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1456" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1456" t="n">
+        <v>43355516</v>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1457" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D1457" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1457" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1457" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1457" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1457" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1457" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1457" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1457" t="n">
+        <v>43578015</v>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D1458" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1458" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1458" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1458" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1458" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1458" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1458" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1458" t="n">
+        <v>43816536</v>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1459" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1459" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1459" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1459" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1459" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="I1459" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1459" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1459" t="n">
+        <v>43578507</v>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1460" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1460" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1460" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1460" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1460" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1460" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1460" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1460" t="n">
+        <v>44398483</v>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D1461" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1461" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1461" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1461" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1461" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I1461" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J1461" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1461" t="n">
+        <v>36320904</v>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D1462" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1462" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1462" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1462" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1462" t="inlineStr">
+        <is>
+          <t>26/36</t>
+        </is>
+      </c>
+      <c r="I1462" s="5" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="J1462" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1462" t="n">
+        <v>36893841</v>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1463" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1463" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1463" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1463" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1463" t="inlineStr">
+        <is>
+          <t>16/36</t>
+        </is>
+      </c>
+      <c r="I1463" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1463" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1463" t="n">
+        <v>36893915</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1445"/>
+  <autoFilter ref="A1:K1463"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-25)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1463</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1471</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1463"/>
+  <dimension ref="A1:K1471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69236,8 +69236,384 @@
         <v>36893915</v>
       </c>
     </row>
+    <row r="1464">
+      <c r="A1464" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1464" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1464" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1464" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1464" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1464" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1464" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1464" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1464" t="n">
+        <v>36323288</v>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1465" t="inlineStr">
+        <is>
+          <t>Guided Session (English version)</t>
+        </is>
+      </c>
+      <c r="E1465" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1465" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1465" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1465" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1465" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1465" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1465" t="n">
+        <v>36323134</v>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1466" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1466" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1466" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1466" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1466" t="inlineStr">
+        <is>
+          <t>10/36</t>
+        </is>
+      </c>
+      <c r="I1466" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1466" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1466" t="n">
+        <v>38771786</v>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1467" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1467" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1467" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1467" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1467" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I1467" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1467" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1467" t="n">
+        <v>36329216</v>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1468" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1468" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1468" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1468" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1468" t="inlineStr">
+        <is>
+          <t>28/36</t>
+        </is>
+      </c>
+      <c r="I1468" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J1468" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1468" t="n">
+        <v>38771886</v>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1469" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1469" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1469" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1469" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1469" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I1469" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J1469" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1469" t="n">
+        <v>36329981</v>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1470" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1470" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1470" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1470" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1470" t="inlineStr">
+        <is>
+          <t>21/36</t>
+        </is>
+      </c>
+      <c r="I1470" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="J1470" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1470" t="n">
+        <v>36323873</v>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>Samedi</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1471" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1471" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1471" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1471" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1471" t="inlineStr">
+        <is>
+          <t>5/36</t>
+        </is>
+      </c>
+      <c r="I1471" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="J1471" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1471" t="n">
+        <v>36935888</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1463"/>
+  <autoFilter ref="A1:K1471"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-26)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1471</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1479</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1471"/>
+  <dimension ref="A1:K1479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69612,8 +69612,384 @@
         <v>36935888</v>
       </c>
     </row>
+    <row r="1472">
+      <c r="A1472" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1472" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1472" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1472" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1472" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1472" t="inlineStr">
+        <is>
+          <t>7/36</t>
+        </is>
+      </c>
+      <c r="I1472" s="4" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="J1472" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1472" t="n">
+        <v>37240298</v>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D1473" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1473" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1473" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1473" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1473" t="inlineStr">
+        <is>
+          <t>14/28</t>
+        </is>
+      </c>
+      <c r="I1473" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1473" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1473" t="n">
+        <v>36336044</v>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B1474" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1474" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D1474" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1474" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1474" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1474" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1474" t="inlineStr">
+        <is>
+          <t>17/36</t>
+        </is>
+      </c>
+      <c r="I1474" s="4" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="J1474" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1474" t="n">
+        <v>37240441</v>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1475" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1475" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1475" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1475" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1475" t="inlineStr">
+        <is>
+          <t>31/36</t>
+        </is>
+      </c>
+      <c r="I1475" s="3" t="n">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="J1475" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1475" t="n">
+        <v>36892158</v>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B1476" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1476" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1476" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1476" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1476" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1476" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1476" t="inlineStr">
+        <is>
+          <t>29/28</t>
+        </is>
+      </c>
+      <c r="I1476" s="3" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="J1476" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1476" t="n">
+        <v>36336259</v>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B1477" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1477" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D1477" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1477" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1477" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1477" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1477" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1477" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1477" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1477" t="n">
+        <v>36692771</v>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B1478" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1478" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="D1478" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1478" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1478" t="n">
+        <v>37</v>
+      </c>
+      <c r="G1478" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1478" t="inlineStr">
+        <is>
+          <t>37/36</t>
+        </is>
+      </c>
+      <c r="I1478" s="3" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="J1478" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1478" t="n">
+        <v>42481099</v>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B1479" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1479" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D1479" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1479" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1479" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1479" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1479" t="inlineStr">
+        <is>
+          <t>5/36</t>
+        </is>
+      </c>
+      <c r="I1479" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="J1479" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1479" t="n">
+        <v>36892113</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1471"/>
+  <autoFilter ref="A1:K1479"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-27)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1479</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1492</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1479"/>
+  <dimension ref="A1:K1492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69988,8 +69988,619 @@
         <v>36892113</v>
       </c>
     </row>
+    <row r="1480">
+      <c r="A1480" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1480" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1480" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1480" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1480" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1480" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1480" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1480" t="inlineStr">
+        <is>
+          <t>1/24</t>
+        </is>
+      </c>
+      <c r="I1480" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="J1480" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1480" t="n">
+        <v>43815080</v>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1481" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1481" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1481" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1481" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1481" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1481" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1481" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1481" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1481" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1481" t="n">
+        <v>43815255</v>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1482" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1482" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1482" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1482" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1482" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1482" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1482" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1482" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1482" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1482" t="n">
+        <v>43815370</v>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1483" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1483" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1483" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1483" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1483" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1483" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1483" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1483" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1483" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1483" t="n">
+        <v>43815395</v>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1484" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1484" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1484" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1484" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1484" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1484" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1484" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1484" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1484" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1484" t="n">
+        <v>43815420</v>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1485" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1485" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1485" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1485" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1485" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1485" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1485" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1485" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1485" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1485" t="n">
+        <v>36390345</v>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1486" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1486" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1486" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1486" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1486" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1486" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1486" t="inlineStr">
+        <is>
+          <t>4/28</t>
+        </is>
+      </c>
+      <c r="I1486" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1486" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1486" t="n">
+        <v>36281148</v>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1487" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1487" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1487" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1487" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1487" t="n">
+        <v>11</v>
+      </c>
+      <c r="G1487" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1487" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I1487" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="J1487" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1487" t="n">
+        <v>38531924</v>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1488" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1488" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1488" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1488" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1488" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1488" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1488" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I1488" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1488" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1488" t="n">
+        <v>36928743</v>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1489" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1489" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1489" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1489" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1489" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1489" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1489" t="inlineStr">
+        <is>
+          <t>24/28</t>
+        </is>
+      </c>
+      <c r="I1489" s="3" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="J1489" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1489" t="n">
+        <v>36281012</v>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1490" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1490" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1490" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1490" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1490" t="n">
+        <v>24</v>
+      </c>
+      <c r="G1490" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1490" t="inlineStr">
+        <is>
+          <t>24/28</t>
+        </is>
+      </c>
+      <c r="I1490" s="3" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="J1490" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1490" t="n">
+        <v>37873154</v>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1491" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1491" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1491" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1491" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1491" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1491" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1491" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1491" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1491" t="n">
+        <v>36929049</v>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B1492" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1492" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1492" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1492" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1492" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1492" t="inlineStr">
+        <is>
+          <t>10/34</t>
+        </is>
+      </c>
+      <c r="I1492" s="4" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="J1492" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1492" t="n">
+        <v>43379264</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1479"/>
+  <autoFilter ref="A1:K1492"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-28)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1492</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1498</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1492"/>
+  <dimension ref="A1:K1498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -70599,8 +70599,290 @@
         <v>43379264</v>
       </c>
     </row>
+    <row r="1493">
+      <c r="A1493" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1493" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1493" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1493" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1493" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1493" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1493" t="inlineStr">
+        <is>
+          <t>5/28</t>
+        </is>
+      </c>
+      <c r="I1493" s="4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="J1493" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1493" t="n">
+        <v>36321376</v>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1494" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D1494" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1494" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1494" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1494" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1494" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I1494" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J1494" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1494" t="n">
+        <v>40188428</v>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1495" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1495" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1495" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1495" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1495" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1495" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I1495" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J1495" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1495" t="n">
+        <v>36929175</v>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1496" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1496" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1496" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1496" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1496" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1496" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="I1496" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J1496" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1496" t="n">
+        <v>36298255</v>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1497" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1497" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1497" t="inlineStr">
+        <is>
+          <t>David Bertin</t>
+        </is>
+      </c>
+      <c r="F1497" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1497" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1497" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I1497" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J1497" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1497" t="n">
+        <v>36297700</v>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B1498" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1498" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1498" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1498" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1498" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1498" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I1498" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J1498" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1498" t="n">
+        <v>36298062</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1492"/>
+  <autoFilter ref="A1:K1498"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-29)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1498</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1505</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1498"/>
+  <dimension ref="A1:K1505"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -70881,8 +70881,337 @@
         <v>36298062</v>
       </c>
     </row>
+    <row r="1499">
+      <c r="A1499" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1499" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1499" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1499" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1499" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1499" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1499" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I1499" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1499" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1499" t="n">
+        <v>36321425</v>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1500" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1500" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1500" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1500" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1500" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1500" t="inlineStr">
+        <is>
+          <t>16/18</t>
+        </is>
+      </c>
+      <c r="I1500" s="3" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="J1500" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1500" t="n">
+        <v>36929307</v>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1501" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1501" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1501" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1501" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1501" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1501" t="inlineStr">
+        <is>
+          <t>13/18</t>
+        </is>
+      </c>
+      <c r="I1501" s="5" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="J1501" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1501" t="n">
+        <v>36298356</v>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1502" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1502" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1502" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1502" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F1502" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1502" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1502" t="inlineStr">
+        <is>
+          <t>26/28</t>
+        </is>
+      </c>
+      <c r="I1502" s="3" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="J1502" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1502" t="n">
+        <v>36298397</v>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1503" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1503" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1503" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1503" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1503" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1503" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1503" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1503" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1503" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1503" t="n">
+        <v>36298594</v>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1504" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1504" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1504" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1504" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1504" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1504" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1504" t="inlineStr">
+        <is>
+          <t>9/8</t>
+        </is>
+      </c>
+      <c r="I1504" s="3" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="J1504" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1504" t="n">
+        <v>40189921</v>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B1505" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1505" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1505" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1505" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1505" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1505" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1505" t="inlineStr">
+        <is>
+          <t>3/34</t>
+        </is>
+      </c>
+      <c r="I1505" s="4" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="J1505" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1505" t="n">
+        <v>43379266</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1498"/>
+  <autoFilter ref="A1:K1505"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-30)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1505</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1519</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1505"/>
+  <dimension ref="A1:K1519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -71210,8 +71210,666 @@
         <v>43379266</v>
       </c>
     </row>
+    <row r="1506">
+      <c r="A1506" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1506" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1506" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1506" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1506" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1506" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1506" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1506" t="inlineStr">
+        <is>
+          <t>7/28</t>
+        </is>
+      </c>
+      <c r="I1506" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1506" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1506" t="n">
+        <v>37090021</v>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1507" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1507" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D1507" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1507" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1507" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1507" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1507" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1507" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1507" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1507" t="n">
+        <v>42435136</v>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1508" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1508" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1508" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1508" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1508" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1508" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1508" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1508" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1508" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1508" t="n">
+        <v>37230129</v>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1509" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1509" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1509" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1509" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1509" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1509" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1509" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1509" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1509" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1509" t="n">
+        <v>37230165</v>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1510" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1510" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1510" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1510" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1510" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1510" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1510" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1510" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1510" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1510" t="n">
+        <v>37090979</v>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1511" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1511" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1511" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1511" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1511" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1511" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1511" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1511" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1511" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1511" t="n">
+        <v>42430596</v>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1512" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1512" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1512" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1512" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1512" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1512" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1512" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1512" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1512" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1512" t="n">
+        <v>42431399</v>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1513" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1513" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1513" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1513" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1513" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1513" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1513" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I1513" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1513" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1513" t="n">
+        <v>36321576</v>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1514" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1514" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1514" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1514" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1514" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1514" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1514" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
+      </c>
+      <c r="I1514" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J1514" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1514" t="n">
+        <v>36929398</v>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1515" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1515" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1515" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1515" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1515" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1515" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1515" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I1515" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1515" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1515" t="n">
+        <v>36298771</v>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1516" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1516" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D1516" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1516" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1516" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1516" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1516" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I1516" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J1516" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1516" t="n">
+        <v>36298825</v>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1517" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1517" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="D1517" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1517" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1517" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1517" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1517" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1517" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1517" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1517" t="n">
+        <v>36298878</v>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1518" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1518" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1518" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1518" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1518" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1518" t="n">
+        <v>8</v>
+      </c>
+      <c r="H1518" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="I1518" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1518" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1518" t="n">
+        <v>40190145</v>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B1519" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1519" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="D1519" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1519" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1519" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1519" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1519" t="inlineStr">
+        <is>
+          <t>4/34</t>
+        </is>
+      </c>
+      <c r="I1519" s="4" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="J1519" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1519" t="n">
+        <v>43379267</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1505"/>
+  <autoFilter ref="A1:K1519"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-10-31)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1519</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1537</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1519"/>
+  <dimension ref="A1:K1537"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -71868,8 +71868,854 @@
         <v>43379267</v>
       </c>
     </row>
+    <row r="1520">
+      <c r="A1520" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1520" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1520" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D1520" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1520" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1520" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1520" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1520" t="inlineStr">
+        <is>
+          <t>3/24</t>
+        </is>
+      </c>
+      <c r="I1520" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J1520" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1520" t="n">
+        <v>43815506</v>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1521" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1521" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1521" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1521" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1521" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1521" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1521" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1521" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1521" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1521" t="n">
+        <v>43815548</v>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1522" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1522" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1522" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1522" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1522" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1522" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1522" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1522" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1522" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1522" t="n">
+        <v>43815645</v>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1523" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1523" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1523" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1523" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1523" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1523" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1523" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1523" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1523" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1523" t="n">
+        <v>43815669</v>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1524" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1524" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1524" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1524" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1524" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1524" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1524" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1524" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1524" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1524" t="n">
+        <v>43816189</v>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1525" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1525" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1525" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1525" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1525" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1525" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1525" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1525" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1525" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1525" t="n">
+        <v>44371084</v>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1526" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1526" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1526" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1526" t="inlineStr">
+        <is>
+          <t>Sigga Daregard</t>
+        </is>
+      </c>
+      <c r="F1526" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1526" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1526" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I1526" s="4" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J1526" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1526" t="n">
+        <v>36319514</v>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1527" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1527" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1527" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1527" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1527" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1527" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1527" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="I1527" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1527" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1527" t="n">
+        <v>36320071</v>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1528" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1528" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D1528" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1528" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1528" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1528" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1528" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1528" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1528" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1528" t="n">
+        <v>36320672</v>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1529" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1529" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D1529" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1529" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1529" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1529" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1529" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1529" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1529" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1529" t="n">
+        <v>44345197</v>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1530" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1530" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D1530" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1530" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1530" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1530" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1530" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1530" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1530" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1530" t="n">
+        <v>43355517</v>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1531" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1531" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D1531" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1531" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1531" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1531" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1531" t="inlineStr">
+        <is>
+          <t>5/10</t>
+        </is>
+      </c>
+      <c r="I1531" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1531" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1531" t="n">
+        <v>43578016</v>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1532" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1532" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D1532" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1532" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1532" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1532" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1532" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1532" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1532" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1532" t="n">
+        <v>43816537</v>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1533" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1533" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1533" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1533" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1533" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1533" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1533" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+      <c r="I1533" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1533" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1533" t="n">
+        <v>43578508</v>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1534" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1534" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1534" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1534" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1534" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1534" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1534" t="inlineStr">
+        <is>
+          <t>5/10</t>
+        </is>
+      </c>
+      <c r="I1534" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1534" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1534" t="n">
+        <v>44576720</v>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1535" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1535" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D1535" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1535" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1535" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1535" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1535" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I1535" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1535" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1535" t="n">
+        <v>36320905</v>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1536" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1536" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D1536" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1536" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1536" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1536" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1536" t="inlineStr">
+        <is>
+          <t>20/36</t>
+        </is>
+      </c>
+      <c r="I1536" s="5" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="J1536" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1536" t="n">
+        <v>36893842</v>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B1537" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1537" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1537" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1537" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1537" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1537" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1537" t="inlineStr">
+        <is>
+          <t>8/36</t>
+        </is>
+      </c>
+      <c r="I1537" s="4" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="J1537" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1537" t="n">
+        <v>36893917</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1519"/>
+  <autoFilter ref="A1:K1537"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>